<commit_message>
[41000013] 配置：更新 AgencyBuilding 建筑表
- 更新 Holmas_AgencyBuildingTable 原始配置表
- 排除 Excel 临时锁文件，避免提交本地编辑副产物
</commit_message>
<xml_diff>
--- a/Assets/Config/Holmas_AgencyBuildingTable.xlsx
+++ b/Assets/Config/Holmas_AgencyBuildingTable.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub\Holmas\Assets\Config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBA46918-7FAF-4240-8818-3361962556C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5BD2BCF-2B03-4967-8C61-005437787317}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -51,9 +51,6 @@
     <t>agencyStageId</t>
   </si>
   <si>
-    <t>stageName</t>
-  </si>
-  <si>
     <t>promotionIds</t>
   </si>
   <si>
@@ -417,10 +414,6 @@
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
   <si>
-    <t>leaflet;radio;tv</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
     <t>柳溪村</t>
   </si>
   <si>
@@ -1038,6 +1031,14 @@
   </si>
   <si>
     <t>城市阶段id</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>leaflet;radio;net</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>stageName</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
 </sst>
@@ -2003,13 +2004,13 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="B1" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="C1" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="D1" t="s">
         <v>0</v>
@@ -2029,2322 +2030,2322 @@
         <v>4</v>
       </c>
       <c r="B2" t="s">
+        <v>331</v>
+      </c>
+      <c r="C2" t="s">
+        <v>317</v>
+      </c>
+      <c r="D2" t="s">
         <v>5</v>
       </c>
-      <c r="C2" t="s">
-        <v>319</v>
-      </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>6</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>7</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>8</v>
-      </c>
-      <c r="G2" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C3" t="s">
+        <v>318</v>
+      </c>
+      <c r="D3" t="s">
+        <v>330</v>
+      </c>
+      <c r="E3" t="s">
+        <v>122</v>
+      </c>
+      <c r="F3" t="s">
+        <v>113</v>
+      </c>
+      <c r="G3" t="s">
         <v>10</v>
-      </c>
-      <c r="B3" t="s">
-        <v>127</v>
-      </c>
-      <c r="C3" t="s">
-        <v>320</v>
-      </c>
-      <c r="D3" t="s">
-        <v>126</v>
-      </c>
-      <c r="E3" t="s">
-        <v>123</v>
-      </c>
-      <c r="F3" t="s">
-        <v>114</v>
-      </c>
-      <c r="G3" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B4" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C4" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="D4" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E4" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F4" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="G4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B5" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="C5" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="D5" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F5" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="G5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B6" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="C6" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="D6" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E6" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F6" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B7" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="C7" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="D7" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E7" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="G7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B8" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C8" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="D8" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E8" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F8" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="G8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B9" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C9" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="D9" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E9" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F9" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="G9" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B10" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="C10" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="D10" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E10" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F10" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="G10" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B11" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C11" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="D11" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E11" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F11" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="G11" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B12" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C12" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="D12" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E12" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F12" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="G12" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B13" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="C13" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="D13" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E13" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F13" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="G13" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B14" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="C14" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="D14" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E14" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F14" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="G14" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B15" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C15" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="D15" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F15" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="G15" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B16" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="C16" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="D16" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E16" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F16" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="G16" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B17" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="C17" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="D17" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E17" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F17" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="G17" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B18" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="C18" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="D18" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E18" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F18" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="G18" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B19" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C19" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="D19" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E19" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F19" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="G19" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B20" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C20" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="D20" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E20" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F20" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="G20" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B21" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="C21" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="D21" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E21" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F21" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="G21" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B22" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="C22" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="D22" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E22" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F22" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="G22" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
+        <v>30</v>
+      </c>
+      <c r="B23" t="s">
+        <v>145</v>
+      </c>
+      <c r="C23" t="s">
+        <v>318</v>
+      </c>
+      <c r="D23" t="s">
+        <v>330</v>
+      </c>
+      <c r="E23" t="s">
+        <v>124</v>
+      </c>
+      <c r="F23" t="s">
+        <v>118</v>
+      </c>
+      <c r="G23" t="s">
         <v>31</v>
-      </c>
-      <c r="B23" t="s">
-        <v>147</v>
-      </c>
-      <c r="C23" t="s">
-        <v>320</v>
-      </c>
-      <c r="D23" t="s">
-        <v>126</v>
-      </c>
-      <c r="E23" t="s">
-        <v>125</v>
-      </c>
-      <c r="F23" t="s">
-        <v>119</v>
-      </c>
-      <c r="G23" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B24" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C24" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="D24" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E24" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F24" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="G24" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B25" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C25" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="D25" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E25" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F25" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="G25" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B26" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C26" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="D26" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E26" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F26" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="G26" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B27" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="C27" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="D27" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E27" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F27" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="G27" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B28" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="C28" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="D28" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E28" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F28" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="G28" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B29" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C29" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="D29" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E29" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F29" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="G29" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B30" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="C30" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="D30" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E30" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F30" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="G30" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B31" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="C31" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="D31" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E31" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F31" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="G31" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B32" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C32" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="D32" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E32" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F32" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="G32" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B33" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C33" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="D33" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E33" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F33" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="G33" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B34" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="C34" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="D34" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E34" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F34" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="G34" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B35" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="C35" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="D35" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E35" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F35" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="G35" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B36" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="C36" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="D36" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E36" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F36" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="G36" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B37" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C37" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="D37" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E37" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F37" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="G37" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B38" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="C38" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="D38" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E38" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F38" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="G38" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B39" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C39" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="D39" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E39" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F39" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="G39" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B40" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="C40" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="D40" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E40" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F40" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="G40" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B41" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="C41" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="D41" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E41" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F41" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="G41" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B42" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="C42" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="D42" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E42" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F42" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="G42" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B43" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C43" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="D43" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E43" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F43" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="G43" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B44" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="C44" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="D44" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E44" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F44" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="G44" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B45" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="C45" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="D45" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E45" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F45" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="G45" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B46" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C46" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="D46" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E46" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F46" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="G46" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B47" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="C47" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="D47" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E47" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F47" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="G47" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B48" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="C48" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="D48" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E48" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F48" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="G48" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B49" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="C49" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="D49" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E49" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F49" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G49" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B50" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="C50" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="D50" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E50" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F50" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="G50" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B51" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="C51" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="D51" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F51" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="G51" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B52" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="C52" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="D52" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E52" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F52" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="G52" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
+        <v>61</v>
+      </c>
+      <c r="B53" t="s">
+        <v>175</v>
+      </c>
+      <c r="C53" t="s">
+        <v>318</v>
+      </c>
+      <c r="D53" t="s">
+        <v>330</v>
+      </c>
+      <c r="E53" t="s">
+        <v>124</v>
+      </c>
+      <c r="F53" t="s">
+        <v>268</v>
+      </c>
+      <c r="G53" t="s">
         <v>62</v>
-      </c>
-      <c r="B53" t="s">
-        <v>177</v>
-      </c>
-      <c r="C53" t="s">
-        <v>320</v>
-      </c>
-      <c r="D53" t="s">
-        <v>126</v>
-      </c>
-      <c r="E53" t="s">
-        <v>125</v>
-      </c>
-      <c r="F53" t="s">
-        <v>270</v>
-      </c>
-      <c r="G53" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B54" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="C54" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="D54" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E54" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F54" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="G54" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B55" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="C55" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="D55" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E55" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F55" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="G55" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B56" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="C56" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="D56" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E56" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F56" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="G56" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B57" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="C57" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="D57" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E57" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F57" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="G57" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B58" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="C58" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="D58" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E58" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F58" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="G58" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B59" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="C59" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="D59" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E59" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F59" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="G59" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B60" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="C60" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="D60" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E60" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F60" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="G60" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B61" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="C61" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="D61" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E61" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F61" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="G61" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B62" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="C62" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="D62" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E62" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F62" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="G62" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B63" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="C63" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="D63" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E63" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F63" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="G63" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B64" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="C64" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="D64" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E64" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F64" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="G64" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B65" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C65" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="D65" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E65" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F65" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="G65" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B66" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C66" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="D66" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E66" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F66" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="G66" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B67" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="C67" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="D67" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E67" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F67" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="G67" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B68" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="C68" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="D68" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E68" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F68" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="G68" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B69" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="C69" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="D69" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E69" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F69" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="G69" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B70" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C70" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="D70" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E70" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F70" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="G70" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B71" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C71" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="D71" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E71" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F71" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="G71" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B72" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C72" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="D72" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E72" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F72" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="G72" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B73" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C73" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="D73" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E73" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F73" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="G73" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B74" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="C74" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="D74" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E74" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F74" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="G74" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B75" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="C75" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="D75" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E75" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F75" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="G75" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B76" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="C76" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="D76" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E76" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F76" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="G76" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B77" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="C77" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="D77" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E77" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F77" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G77" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B78" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="C78" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="D78" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E78" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F78" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="G78" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B79" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="C79" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="D79" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E79" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F79" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="G79" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B80" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="C80" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="D80" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E80" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F80" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="G80" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B81" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="C81" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="D81" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E81" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F81" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="G81" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B82" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="C82" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="D82" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E82" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F82" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="G82" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
+        <v>92</v>
+      </c>
+      <c r="B83" t="s">
+        <v>205</v>
+      </c>
+      <c r="C83" t="s">
+        <v>318</v>
+      </c>
+      <c r="D83" t="s">
+        <v>330</v>
+      </c>
+      <c r="E83" t="s">
+        <v>124</v>
+      </c>
+      <c r="F83" t="s">
+        <v>296</v>
+      </c>
+      <c r="G83" t="s">
         <v>93</v>
-      </c>
-      <c r="B83" t="s">
-        <v>207</v>
-      </c>
-      <c r="C83" t="s">
-        <v>320</v>
-      </c>
-      <c r="D83" t="s">
-        <v>126</v>
-      </c>
-      <c r="E83" t="s">
-        <v>125</v>
-      </c>
-      <c r="F83" t="s">
-        <v>298</v>
-      </c>
-      <c r="G83" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B84" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="C84" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="D84" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E84" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F84" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="G84" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="85" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B85" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="C85" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="D85" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E85" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F85" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="G85" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="86" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B86" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="C86" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="D86" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E86" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F86" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="G86" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B87" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="C87" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="D87" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E87" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F87" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="G87" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B88" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="C88" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="D88" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E88" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F88" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="G88" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B89" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="C89" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="D89" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E89" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F89" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="G89" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B90" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="C90" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="D90" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E90" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F90" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="G90" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="91" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B91" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="C91" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="D91" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E91" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F91" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="G91" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B92" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="C92" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="D92" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E92" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F92" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="G92" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="93" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B93" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="C93" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="D93" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E93" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F93" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="G93" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="94" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B94" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="C94" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="D94" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E94" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F94" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="G94" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="95" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B95" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="C95" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="D95" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E95" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F95" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="G95" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="96" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B96" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="C96" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="D96" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E96" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F96" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="G96" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="97" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B97" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="C97" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="D97" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E97" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F97" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="G97" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="98" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B98" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="C98" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="D98" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E98" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F98" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="G98" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="99" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B99" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="C99" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="D99" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E99" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F99" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="G99" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="100" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B100" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="C100" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="D100" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E100" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F100" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="G100" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B101" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="C101" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="D101" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E101" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F101" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="G101" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="102" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B102" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="C102" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="D102" t="s">
-        <v>126</v>
+        <v>330</v>
       </c>
       <c r="E102" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F102" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="G102" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[41000014] 配置：更新 AgencyBuilding 宣传配置
- 更新 Holmas_AgencyBuildingTable 及导出的核心 JSON/bytes 配置

- 将 AgencyBuilding 宣传项从 tv 调整为 net，并补充 buttonImage 扩展字段

- 刷新配置导出报告时间戳
</commit_message>
<xml_diff>
--- a/Assets/Config/Holmas_AgencyBuildingTable.xlsx
+++ b/Assets/Config/Holmas_AgencyBuildingTable.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub\Holmas\Assets\Config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5BD2BCF-2B03-4967-8C61-005437787317}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6120A236-FFDD-48DD-9E31-91502C2FA7F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="714" uniqueCount="332">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="816" uniqueCount="335">
   <si>
     <t>宣传功能id数组</t>
   </si>
@@ -1039,6 +1039,18 @@
   </si>
   <si>
     <t>stageName</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>宣传按钮图片路劲</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>buttonImage</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>Textures/NewUIRes/leaflet.png;Textures/NewUIRes/radio.png;Textures/NewUIRes/net.png;</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
 </sst>
@@ -1991,18 +2003,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G102"/>
+  <dimension ref="A1:H102"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="16.25" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="29.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20.25" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="73.4140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.6640625" customWidth="1"/>
+    <col min="5" max="5" width="18" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.25" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="73.4140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>329</v>
       </c>
@@ -2013,19 +2026,22 @@
         <v>316</v>
       </c>
       <c r="D1" t="s">
+        <v>332</v>
+      </c>
+      <c r="E1" t="s">
         <v>0</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>1</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>2</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -2036,19 +2052,22 @@
         <v>317</v>
       </c>
       <c r="D2" t="s">
+        <v>333</v>
+      </c>
+      <c r="E2" t="s">
         <v>5</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>6</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>7</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -2059,19 +2078,22 @@
         <v>318</v>
       </c>
       <c r="D3" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E3" t="s">
+        <v>330</v>
+      </c>
+      <c r="F3" t="s">
         <v>122</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>113</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>11</v>
       </c>
@@ -2082,19 +2104,22 @@
         <v>319</v>
       </c>
       <c r="D4" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E4" t="s">
+        <v>330</v>
+      </c>
+      <c r="F4" t="s">
         <v>123</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>114</v>
       </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -2105,19 +2130,22 @@
         <v>320</v>
       </c>
       <c r="D5" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E5" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F5" t="s">
+        <v>124</v>
+      </c>
+      <c r="G5" t="s">
         <v>115</v>
       </c>
-      <c r="G5" t="s">
+      <c r="H5" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>13</v>
       </c>
@@ -2128,19 +2156,22 @@
         <v>321</v>
       </c>
       <c r="D6" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E6" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F6" t="s">
+        <v>124</v>
+      </c>
+      <c r="G6" t="s">
         <v>116</v>
       </c>
-      <c r="G6" t="s">
+      <c r="H6" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>14</v>
       </c>
@@ -2151,19 +2182,22 @@
         <v>322</v>
       </c>
       <c r="D7" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E7" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F7" t="s">
+        <v>124</v>
+      </c>
+      <c r="G7" t="s">
         <v>117</v>
       </c>
-      <c r="G7" t="s">
+      <c r="H7" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>15</v>
       </c>
@@ -2174,19 +2208,22 @@
         <v>323</v>
       </c>
       <c r="D8" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E8" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F8" t="s">
+        <v>124</v>
+      </c>
+      <c r="G8" t="s">
         <v>225</v>
       </c>
-      <c r="G8" t="s">
+      <c r="H8" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>16</v>
       </c>
@@ -2197,19 +2234,22 @@
         <v>324</v>
       </c>
       <c r="D9" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E9" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F9" t="s">
+        <v>124</v>
+      </c>
+      <c r="G9" t="s">
         <v>226</v>
       </c>
-      <c r="G9" t="s">
+      <c r="H9" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>17</v>
       </c>
@@ -2220,19 +2260,22 @@
         <v>325</v>
       </c>
       <c r="D10" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E10" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F10" t="s">
+        <v>124</v>
+      </c>
+      <c r="G10" t="s">
         <v>227</v>
       </c>
-      <c r="G10" t="s">
+      <c r="H10" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>18</v>
       </c>
@@ -2243,19 +2286,22 @@
         <v>326</v>
       </c>
       <c r="D11" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E11" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F11" t="s">
+        <v>124</v>
+      </c>
+      <c r="G11" t="s">
         <v>228</v>
       </c>
-      <c r="G11" t="s">
+      <c r="H11" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>19</v>
       </c>
@@ -2266,19 +2312,22 @@
         <v>327</v>
       </c>
       <c r="D12" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E12" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F12" t="s">
+        <v>124</v>
+      </c>
+      <c r="G12" t="s">
         <v>229</v>
       </c>
-      <c r="G12" t="s">
+      <c r="H12" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>20</v>
       </c>
@@ -2289,19 +2338,22 @@
         <v>318</v>
       </c>
       <c r="D13" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E13" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F13" t="s">
+        <v>124</v>
+      </c>
+      <c r="G13" t="s">
         <v>230</v>
       </c>
-      <c r="G13" t="s">
+      <c r="H13" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>21</v>
       </c>
@@ -2312,19 +2364,22 @@
         <v>319</v>
       </c>
       <c r="D14" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E14" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F14" t="s">
+        <v>124</v>
+      </c>
+      <c r="G14" t="s">
         <v>231</v>
       </c>
-      <c r="G14" t="s">
+      <c r="H14" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>22</v>
       </c>
@@ -2335,19 +2390,22 @@
         <v>320</v>
       </c>
       <c r="D15" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E15" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F15" t="s">
+        <v>124</v>
+      </c>
+      <c r="G15" t="s">
         <v>232</v>
       </c>
-      <c r="G15" t="s">
+      <c r="H15" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>23</v>
       </c>
@@ -2358,19 +2416,22 @@
         <v>321</v>
       </c>
       <c r="D16" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E16" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F16" t="s">
+        <v>124</v>
+      </c>
+      <c r="G16" t="s">
         <v>233</v>
       </c>
-      <c r="G16" t="s">
+      <c r="H16" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>24</v>
       </c>
@@ -2381,19 +2442,22 @@
         <v>322</v>
       </c>
       <c r="D17" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E17" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F17" t="s">
+        <v>124</v>
+      </c>
+      <c r="G17" t="s">
         <v>234</v>
       </c>
-      <c r="G17" t="s">
+      <c r="H17" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>25</v>
       </c>
@@ -2404,19 +2468,22 @@
         <v>323</v>
       </c>
       <c r="D18" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E18" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F18" t="s">
+        <v>124</v>
+      </c>
+      <c r="G18" t="s">
         <v>235</v>
       </c>
-      <c r="G18" t="s">
+      <c r="H18" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>26</v>
       </c>
@@ -2427,19 +2494,22 @@
         <v>324</v>
       </c>
       <c r="D19" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E19" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F19" t="s">
+        <v>124</v>
+      </c>
+      <c r="G19" t="s">
         <v>236</v>
       </c>
-      <c r="G19" t="s">
+      <c r="H19" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>27</v>
       </c>
@@ -2450,19 +2520,22 @@
         <v>325</v>
       </c>
       <c r="D20" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E20" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F20" t="s">
+        <v>124</v>
+      </c>
+      <c r="G20" t="s">
         <v>237</v>
       </c>
-      <c r="G20" t="s">
+      <c r="H20" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>28</v>
       </c>
@@ -2473,19 +2546,22 @@
         <v>326</v>
       </c>
       <c r="D21" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E21" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F21" t="s">
+        <v>124</v>
+      </c>
+      <c r="G21" t="s">
         <v>238</v>
       </c>
-      <c r="G21" t="s">
+      <c r="H21" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>29</v>
       </c>
@@ -2496,19 +2572,22 @@
         <v>327</v>
       </c>
       <c r="D22" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E22" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F22" t="s">
+        <v>124</v>
+      </c>
+      <c r="G22" t="s">
         <v>239</v>
       </c>
-      <c r="G22" t="s">
+      <c r="H22" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>30</v>
       </c>
@@ -2519,19 +2598,22 @@
         <v>318</v>
       </c>
       <c r="D23" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E23" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F23" t="s">
+        <v>124</v>
+      </c>
+      <c r="G23" t="s">
         <v>118</v>
       </c>
-      <c r="G23" t="s">
+      <c r="H23" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>32</v>
       </c>
@@ -2542,19 +2624,22 @@
         <v>319</v>
       </c>
       <c r="D24" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E24" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F24" t="s">
+        <v>124</v>
+      </c>
+      <c r="G24" t="s">
         <v>240</v>
       </c>
-      <c r="G24" t="s">
+      <c r="H24" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>33</v>
       </c>
@@ -2565,19 +2650,22 @@
         <v>320</v>
       </c>
       <c r="D25" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E25" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F25" t="s">
+        <v>124</v>
+      </c>
+      <c r="G25" t="s">
         <v>241</v>
       </c>
-      <c r="G25" t="s">
+      <c r="H25" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>34</v>
       </c>
@@ -2588,19 +2676,22 @@
         <v>321</v>
       </c>
       <c r="D26" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E26" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F26" t="s">
+        <v>124</v>
+      </c>
+      <c r="G26" t="s">
         <v>242</v>
       </c>
-      <c r="G26" t="s">
+      <c r="H26" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>35</v>
       </c>
@@ -2611,19 +2702,22 @@
         <v>322</v>
       </c>
       <c r="D27" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E27" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F27" t="s">
+        <v>124</v>
+      </c>
+      <c r="G27" t="s">
         <v>243</v>
       </c>
-      <c r="G27" t="s">
+      <c r="H27" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>36</v>
       </c>
@@ -2634,19 +2728,22 @@
         <v>323</v>
       </c>
       <c r="D28" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E28" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F28" t="s">
+        <v>124</v>
+      </c>
+      <c r="G28" t="s">
         <v>244</v>
       </c>
-      <c r="G28" t="s">
+      <c r="H28" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>37</v>
       </c>
@@ -2657,19 +2754,22 @@
         <v>324</v>
       </c>
       <c r="D29" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E29" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F29" t="s">
+        <v>124</v>
+      </c>
+      <c r="G29" t="s">
         <v>245</v>
       </c>
-      <c r="G29" t="s">
+      <c r="H29" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>38</v>
       </c>
@@ -2680,19 +2780,22 @@
         <v>325</v>
       </c>
       <c r="D30" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E30" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F30" t="s">
+        <v>124</v>
+      </c>
+      <c r="G30" t="s">
         <v>246</v>
       </c>
-      <c r="G30" t="s">
+      <c r="H30" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>39</v>
       </c>
@@ -2703,19 +2806,22 @@
         <v>326</v>
       </c>
       <c r="D31" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E31" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F31" t="s">
+        <v>124</v>
+      </c>
+      <c r="G31" t="s">
         <v>247</v>
       </c>
-      <c r="G31" t="s">
+      <c r="H31" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>40</v>
       </c>
@@ -2726,19 +2832,22 @@
         <v>327</v>
       </c>
       <c r="D32" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E32" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F32" t="s">
+        <v>124</v>
+      </c>
+      <c r="G32" t="s">
         <v>248</v>
       </c>
-      <c r="G32" t="s">
+      <c r="H32" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>41</v>
       </c>
@@ -2749,19 +2858,22 @@
         <v>318</v>
       </c>
       <c r="D33" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E33" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F33" t="s">
+        <v>124</v>
+      </c>
+      <c r="G33" t="s">
         <v>249</v>
       </c>
-      <c r="G33" t="s">
+      <c r="H33" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>42</v>
       </c>
@@ -2772,19 +2884,22 @@
         <v>319</v>
       </c>
       <c r="D34" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E34" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F34" t="s">
+        <v>124</v>
+      </c>
+      <c r="G34" t="s">
         <v>250</v>
       </c>
-      <c r="G34" t="s">
+      <c r="H34" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>43</v>
       </c>
@@ -2795,19 +2910,22 @@
         <v>320</v>
       </c>
       <c r="D35" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E35" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F35" t="s">
+        <v>124</v>
+      </c>
+      <c r="G35" t="s">
         <v>251</v>
       </c>
-      <c r="G35" t="s">
+      <c r="H35" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>44</v>
       </c>
@@ -2818,19 +2936,22 @@
         <v>321</v>
       </c>
       <c r="D36" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E36" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F36" t="s">
+        <v>124</v>
+      </c>
+      <c r="G36" t="s">
         <v>252</v>
       </c>
-      <c r="G36" t="s">
+      <c r="H36" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>45</v>
       </c>
@@ -2841,19 +2962,22 @@
         <v>322</v>
       </c>
       <c r="D37" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E37" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F37" t="s">
+        <v>124</v>
+      </c>
+      <c r="G37" t="s">
         <v>253</v>
       </c>
-      <c r="G37" t="s">
+      <c r="H37" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>46</v>
       </c>
@@ -2864,19 +2988,22 @@
         <v>323</v>
       </c>
       <c r="D38" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E38" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F38" t="s">
+        <v>124</v>
+      </c>
+      <c r="G38" t="s">
         <v>254</v>
       </c>
-      <c r="G38" t="s">
+      <c r="H38" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>47</v>
       </c>
@@ -2887,19 +3014,22 @@
         <v>324</v>
       </c>
       <c r="D39" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E39" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F39" t="s">
+        <v>124</v>
+      </c>
+      <c r="G39" t="s">
         <v>255</v>
       </c>
-      <c r="G39" t="s">
+      <c r="H39" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>48</v>
       </c>
@@ -2910,19 +3040,22 @@
         <v>325</v>
       </c>
       <c r="D40" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E40" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F40" t="s">
+        <v>124</v>
+      </c>
+      <c r="G40" t="s">
         <v>256</v>
       </c>
-      <c r="G40" t="s">
+      <c r="H40" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>49</v>
       </c>
@@ -2933,19 +3066,22 @@
         <v>326</v>
       </c>
       <c r="D41" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E41" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F41" t="s">
+        <v>124</v>
+      </c>
+      <c r="G41" t="s">
         <v>257</v>
       </c>
-      <c r="G41" t="s">
+      <c r="H41" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>50</v>
       </c>
@@ -2956,19 +3092,22 @@
         <v>327</v>
       </c>
       <c r="D42" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E42" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F42" t="s">
+        <v>124</v>
+      </c>
+      <c r="G42" t="s">
         <v>258</v>
       </c>
-      <c r="G42" t="s">
+      <c r="H42" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>51</v>
       </c>
@@ -2979,19 +3118,22 @@
         <v>318</v>
       </c>
       <c r="D43" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E43" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F43" t="s">
+        <v>124</v>
+      </c>
+      <c r="G43" t="s">
         <v>259</v>
       </c>
-      <c r="G43" t="s">
+      <c r="H43" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>52</v>
       </c>
@@ -3002,19 +3144,22 @@
         <v>319</v>
       </c>
       <c r="D44" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E44" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F44" t="s">
+        <v>124</v>
+      </c>
+      <c r="G44" t="s">
         <v>260</v>
       </c>
-      <c r="G44" t="s">
+      <c r="H44" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>53</v>
       </c>
@@ -3025,19 +3170,22 @@
         <v>320</v>
       </c>
       <c r="D45" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E45" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F45" t="s">
+        <v>124</v>
+      </c>
+      <c r="G45" t="s">
         <v>261</v>
       </c>
-      <c r="G45" t="s">
+      <c r="H45" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>54</v>
       </c>
@@ -3048,19 +3196,22 @@
         <v>321</v>
       </c>
       <c r="D46" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E46" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F46" t="s">
+        <v>124</v>
+      </c>
+      <c r="G46" t="s">
         <v>262</v>
       </c>
-      <c r="G46" t="s">
+      <c r="H46" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>55</v>
       </c>
@@ -3071,19 +3222,22 @@
         <v>322</v>
       </c>
       <c r="D47" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E47" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F47" t="s">
+        <v>124</v>
+      </c>
+      <c r="G47" t="s">
         <v>263</v>
       </c>
-      <c r="G47" t="s">
+      <c r="H47" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>56</v>
       </c>
@@ -3094,19 +3248,22 @@
         <v>323</v>
       </c>
       <c r="D48" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E48" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F48" t="s">
+        <v>124</v>
+      </c>
+      <c r="G48" t="s">
         <v>264</v>
       </c>
-      <c r="G48" t="s">
+      <c r="H48" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>57</v>
       </c>
@@ -3117,19 +3274,22 @@
         <v>324</v>
       </c>
       <c r="D49" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E49" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F49" t="s">
+        <v>124</v>
+      </c>
+      <c r="G49" t="s">
         <v>119</v>
       </c>
-      <c r="G49" t="s">
+      <c r="H49" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>58</v>
       </c>
@@ -3140,19 +3300,22 @@
         <v>325</v>
       </c>
       <c r="D50" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E50" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F50" t="s">
+        <v>124</v>
+      </c>
+      <c r="G50" t="s">
         <v>265</v>
       </c>
-      <c r="G50" t="s">
+      <c r="H50" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>59</v>
       </c>
@@ -3163,19 +3326,22 @@
         <v>326</v>
       </c>
       <c r="D51" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E51" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F51" t="s">
+        <v>124</v>
+      </c>
+      <c r="G51" t="s">
         <v>266</v>
       </c>
-      <c r="G51" t="s">
+      <c r="H51" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>60</v>
       </c>
@@ -3186,19 +3352,22 @@
         <v>327</v>
       </c>
       <c r="D52" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E52" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F52" t="s">
+        <v>124</v>
+      </c>
+      <c r="G52" t="s">
         <v>267</v>
       </c>
-      <c r="G52" t="s">
+      <c r="H52" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>61</v>
       </c>
@@ -3209,19 +3378,22 @@
         <v>318</v>
       </c>
       <c r="D53" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E53" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F53" t="s">
+        <v>124</v>
+      </c>
+      <c r="G53" t="s">
         <v>268</v>
       </c>
-      <c r="G53" t="s">
+      <c r="H53" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>63</v>
       </c>
@@ -3232,19 +3404,22 @@
         <v>319</v>
       </c>
       <c r="D54" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E54" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F54" t="s">
+        <v>124</v>
+      </c>
+      <c r="G54" t="s">
         <v>269</v>
       </c>
-      <c r="G54" t="s">
+      <c r="H54" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>64</v>
       </c>
@@ -3255,19 +3430,22 @@
         <v>320</v>
       </c>
       <c r="D55" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E55" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F55" t="s">
+        <v>124</v>
+      </c>
+      <c r="G55" t="s">
         <v>270</v>
       </c>
-      <c r="G55" t="s">
+      <c r="H55" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>65</v>
       </c>
@@ -3278,19 +3456,22 @@
         <v>321</v>
       </c>
       <c r="D56" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E56" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F56" t="s">
+        <v>124</v>
+      </c>
+      <c r="G56" t="s">
         <v>271</v>
       </c>
-      <c r="G56" t="s">
+      <c r="H56" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>66</v>
       </c>
@@ -3301,19 +3482,22 @@
         <v>322</v>
       </c>
       <c r="D57" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E57" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F57" t="s">
+        <v>124</v>
+      </c>
+      <c r="G57" t="s">
         <v>272</v>
       </c>
-      <c r="G57" t="s">
+      <c r="H57" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>67</v>
       </c>
@@ -3324,19 +3508,22 @@
         <v>323</v>
       </c>
       <c r="D58" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E58" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F58" t="s">
+        <v>124</v>
+      </c>
+      <c r="G58" t="s">
         <v>273</v>
       </c>
-      <c r="G58" t="s">
+      <c r="H58" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>68</v>
       </c>
@@ -3347,19 +3534,22 @@
         <v>324</v>
       </c>
       <c r="D59" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E59" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F59" t="s">
+        <v>124</v>
+      </c>
+      <c r="G59" t="s">
         <v>274</v>
       </c>
-      <c r="G59" t="s">
+      <c r="H59" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>69</v>
       </c>
@@ -3370,19 +3560,22 @@
         <v>325</v>
       </c>
       <c r="D60" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E60" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F60" t="s">
+        <v>124</v>
+      </c>
+      <c r="G60" t="s">
         <v>275</v>
       </c>
-      <c r="G60" t="s">
+      <c r="H60" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>70</v>
       </c>
@@ -3393,19 +3586,22 @@
         <v>326</v>
       </c>
       <c r="D61" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E61" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F61" t="s">
+        <v>124</v>
+      </c>
+      <c r="G61" t="s">
         <v>276</v>
       </c>
-      <c r="G61" t="s">
+      <c r="H61" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>71</v>
       </c>
@@ -3416,19 +3612,22 @@
         <v>327</v>
       </c>
       <c r="D62" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E62" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F62" t="s">
+        <v>124</v>
+      </c>
+      <c r="G62" t="s">
         <v>120</v>
       </c>
-      <c r="G62" t="s">
+      <c r="H62" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>72</v>
       </c>
@@ -3439,19 +3638,22 @@
         <v>318</v>
       </c>
       <c r="D63" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E63" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F63" t="s">
+        <v>124</v>
+      </c>
+      <c r="G63" t="s">
         <v>277</v>
       </c>
-      <c r="G63" t="s">
+      <c r="H63" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>73</v>
       </c>
@@ -3462,19 +3664,22 @@
         <v>319</v>
       </c>
       <c r="D64" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E64" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F64" t="s">
+        <v>124</v>
+      </c>
+      <c r="G64" t="s">
         <v>278</v>
       </c>
-      <c r="G64" t="s">
+      <c r="H64" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>74</v>
       </c>
@@ -3485,19 +3690,22 @@
         <v>320</v>
       </c>
       <c r="D65" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E65" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F65" t="s">
+        <v>124</v>
+      </c>
+      <c r="G65" t="s">
         <v>279</v>
       </c>
-      <c r="G65" t="s">
+      <c r="H65" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>75</v>
       </c>
@@ -3508,19 +3716,22 @@
         <v>321</v>
       </c>
       <c r="D66" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E66" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F66" t="s">
+        <v>124</v>
+      </c>
+      <c r="G66" t="s">
         <v>280</v>
       </c>
-      <c r="G66" t="s">
+      <c r="H66" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>76</v>
       </c>
@@ -3531,19 +3742,22 @@
         <v>322</v>
       </c>
       <c r="D67" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E67" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F67" t="s">
+        <v>124</v>
+      </c>
+      <c r="G67" t="s">
         <v>281</v>
       </c>
-      <c r="G67" t="s">
+      <c r="H67" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>77</v>
       </c>
@@ -3554,19 +3768,22 @@
         <v>323</v>
       </c>
       <c r="D68" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E68" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F68" t="s">
+        <v>124</v>
+      </c>
+      <c r="G68" t="s">
         <v>282</v>
       </c>
-      <c r="G68" t="s">
+      <c r="H68" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>78</v>
       </c>
@@ -3577,19 +3794,22 @@
         <v>324</v>
       </c>
       <c r="D69" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E69" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F69" t="s">
+        <v>124</v>
+      </c>
+      <c r="G69" t="s">
         <v>283</v>
       </c>
-      <c r="G69" t="s">
+      <c r="H69" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>79</v>
       </c>
@@ -3600,19 +3820,22 @@
         <v>325</v>
       </c>
       <c r="D70" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E70" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F70" t="s">
+        <v>124</v>
+      </c>
+      <c r="G70" t="s">
         <v>284</v>
       </c>
-      <c r="G70" t="s">
+      <c r="H70" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>80</v>
       </c>
@@ -3623,19 +3846,22 @@
         <v>326</v>
       </c>
       <c r="D71" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E71" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F71" t="s">
+        <v>124</v>
+      </c>
+      <c r="G71" t="s">
         <v>285</v>
       </c>
-      <c r="G71" t="s">
+      <c r="H71" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>81</v>
       </c>
@@ -3646,19 +3872,22 @@
         <v>327</v>
       </c>
       <c r="D72" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E72" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F72" t="s">
+        <v>124</v>
+      </c>
+      <c r="G72" t="s">
         <v>286</v>
       </c>
-      <c r="G72" t="s">
+      <c r="H72" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>82</v>
       </c>
@@ -3669,19 +3898,22 @@
         <v>318</v>
       </c>
       <c r="D73" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E73" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F73" t="s">
+        <v>124</v>
+      </c>
+      <c r="G73" t="s">
         <v>287</v>
       </c>
-      <c r="G73" t="s">
+      <c r="H73" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>83</v>
       </c>
@@ -3692,19 +3924,22 @@
         <v>319</v>
       </c>
       <c r="D74" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E74" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F74" t="s">
+        <v>124</v>
+      </c>
+      <c r="G74" t="s">
         <v>288</v>
       </c>
-      <c r="G74" t="s">
+      <c r="H74" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>84</v>
       </c>
@@ -3715,19 +3950,22 @@
         <v>320</v>
       </c>
       <c r="D75" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E75" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F75" t="s">
+        <v>124</v>
+      </c>
+      <c r="G75" t="s">
         <v>289</v>
       </c>
-      <c r="G75" t="s">
+      <c r="H75" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>85</v>
       </c>
@@ -3738,19 +3976,22 @@
         <v>321</v>
       </c>
       <c r="D76" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E76" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F76" t="s">
+        <v>124</v>
+      </c>
+      <c r="G76" t="s">
         <v>290</v>
       </c>
-      <c r="G76" t="s">
+      <c r="H76" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>86</v>
       </c>
@@ -3761,19 +4002,22 @@
         <v>322</v>
       </c>
       <c r="D77" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E77" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F77" t="s">
+        <v>124</v>
+      </c>
+      <c r="G77" t="s">
         <v>121</v>
       </c>
-      <c r="G77" t="s">
+      <c r="H77" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>87</v>
       </c>
@@ -3784,19 +4028,22 @@
         <v>323</v>
       </c>
       <c r="D78" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E78" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F78" t="s">
+        <v>124</v>
+      </c>
+      <c r="G78" t="s">
         <v>291</v>
       </c>
-      <c r="G78" t="s">
+      <c r="H78" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>88</v>
       </c>
@@ -3807,19 +4054,22 @@
         <v>324</v>
       </c>
       <c r="D79" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E79" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F79" t="s">
+        <v>124</v>
+      </c>
+      <c r="G79" t="s">
         <v>292</v>
       </c>
-      <c r="G79" t="s">
+      <c r="H79" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>89</v>
       </c>
@@ -3830,19 +4080,22 @@
         <v>325</v>
       </c>
       <c r="D80" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E80" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F80" t="s">
+        <v>124</v>
+      </c>
+      <c r="G80" t="s">
         <v>293</v>
       </c>
-      <c r="G80" t="s">
+      <c r="H80" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>90</v>
       </c>
@@ -3853,19 +4106,22 @@
         <v>326</v>
       </c>
       <c r="D81" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E81" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F81" t="s">
+        <v>124</v>
+      </c>
+      <c r="G81" t="s">
         <v>294</v>
       </c>
-      <c r="G81" t="s">
+      <c r="H81" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>91</v>
       </c>
@@ -3876,19 +4132,22 @@
         <v>327</v>
       </c>
       <c r="D82" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E82" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F82" t="s">
+        <v>124</v>
+      </c>
+      <c r="G82" t="s">
         <v>295</v>
       </c>
-      <c r="G82" t="s">
+      <c r="H82" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>92</v>
       </c>
@@ -3899,19 +4158,22 @@
         <v>318</v>
       </c>
       <c r="D83" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E83" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F83" t="s">
+        <v>124</v>
+      </c>
+      <c r="G83" t="s">
         <v>296</v>
       </c>
-      <c r="G83" t="s">
+      <c r="H83" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>94</v>
       </c>
@@ -3922,19 +4184,22 @@
         <v>319</v>
       </c>
       <c r="D84" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E84" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F84" t="s">
+        <v>124</v>
+      </c>
+      <c r="G84" t="s">
         <v>297</v>
       </c>
-      <c r="G84" t="s">
+      <c r="H84" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>95</v>
       </c>
@@ -3945,19 +4210,22 @@
         <v>320</v>
       </c>
       <c r="D85" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E85" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F85" t="s">
+        <v>124</v>
+      </c>
+      <c r="G85" t="s">
         <v>298</v>
       </c>
-      <c r="G85" t="s">
+      <c r="H85" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>96</v>
       </c>
@@ -3968,19 +4236,22 @@
         <v>321</v>
       </c>
       <c r="D86" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E86" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F86" t="s">
+        <v>124</v>
+      </c>
+      <c r="G86" t="s">
         <v>299</v>
       </c>
-      <c r="G86" t="s">
+      <c r="H86" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>97</v>
       </c>
@@ -3991,19 +4262,22 @@
         <v>322</v>
       </c>
       <c r="D87" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E87" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F87" t="s">
+        <v>124</v>
+      </c>
+      <c r="G87" t="s">
         <v>300</v>
       </c>
-      <c r="G87" t="s">
+      <c r="H87" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>98</v>
       </c>
@@ -4014,19 +4288,22 @@
         <v>323</v>
       </c>
       <c r="D88" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E88" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F88" t="s">
+        <v>124</v>
+      </c>
+      <c r="G88" t="s">
         <v>301</v>
       </c>
-      <c r="G88" t="s">
+      <c r="H88" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>99</v>
       </c>
@@ -4037,19 +4314,22 @@
         <v>324</v>
       </c>
       <c r="D89" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E89" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F89" t="s">
+        <v>124</v>
+      </c>
+      <c r="G89" t="s">
         <v>302</v>
       </c>
-      <c r="G89" t="s">
+      <c r="H89" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>100</v>
       </c>
@@ -4060,19 +4340,22 @@
         <v>325</v>
       </c>
       <c r="D90" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E90" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F90" t="s">
+        <v>124</v>
+      </c>
+      <c r="G90" t="s">
         <v>303</v>
       </c>
-      <c r="G90" t="s">
+      <c r="H90" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>101</v>
       </c>
@@ -4083,19 +4366,22 @@
         <v>326</v>
       </c>
       <c r="D91" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E91" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F91" t="s">
+        <v>124</v>
+      </c>
+      <c r="G91" t="s">
         <v>304</v>
       </c>
-      <c r="G91" t="s">
+      <c r="H91" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>102</v>
       </c>
@@ -4106,19 +4392,22 @@
         <v>327</v>
       </c>
       <c r="D92" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E92" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F92" t="s">
+        <v>124</v>
+      </c>
+      <c r="G92" t="s">
         <v>305</v>
       </c>
-      <c r="G92" t="s">
+      <c r="H92" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>103</v>
       </c>
@@ -4129,19 +4418,22 @@
         <v>318</v>
       </c>
       <c r="D93" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E93" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F93" t="s">
+        <v>124</v>
+      </c>
+      <c r="G93" t="s">
         <v>306</v>
       </c>
-      <c r="G93" t="s">
+      <c r="H93" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>104</v>
       </c>
@@ -4152,19 +4444,22 @@
         <v>319</v>
       </c>
       <c r="D94" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E94" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F94" t="s">
+        <v>124</v>
+      </c>
+      <c r="G94" t="s">
         <v>307</v>
       </c>
-      <c r="G94" t="s">
+      <c r="H94" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>105</v>
       </c>
@@ -4175,19 +4470,22 @@
         <v>320</v>
       </c>
       <c r="D95" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E95" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F95" t="s">
+        <v>124</v>
+      </c>
+      <c r="G95" t="s">
         <v>308</v>
       </c>
-      <c r="G95" t="s">
+      <c r="H95" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>106</v>
       </c>
@@ -4198,19 +4496,22 @@
         <v>321</v>
       </c>
       <c r="D96" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E96" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F96" t="s">
+        <v>124</v>
+      </c>
+      <c r="G96" t="s">
         <v>309</v>
       </c>
-      <c r="G96" t="s">
+      <c r="H96" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>107</v>
       </c>
@@ -4221,19 +4522,22 @@
         <v>322</v>
       </c>
       <c r="D97" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E97" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F97" t="s">
+        <v>124</v>
+      </c>
+      <c r="G97" t="s">
         <v>310</v>
       </c>
-      <c r="G97" t="s">
+      <c r="H97" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>108</v>
       </c>
@@ -4244,19 +4548,22 @@
         <v>323</v>
       </c>
       <c r="D98" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E98" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F98" t="s">
+        <v>124</v>
+      </c>
+      <c r="G98" t="s">
         <v>311</v>
       </c>
-      <c r="G98" t="s">
+      <c r="H98" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>109</v>
       </c>
@@ -4267,19 +4574,22 @@
         <v>324</v>
       </c>
       <c r="D99" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E99" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F99" t="s">
+        <v>124</v>
+      </c>
+      <c r="G99" t="s">
         <v>312</v>
       </c>
-      <c r="G99" t="s">
+      <c r="H99" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>110</v>
       </c>
@@ -4290,19 +4600,22 @@
         <v>325</v>
       </c>
       <c r="D100" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E100" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F100" t="s">
+        <v>124</v>
+      </c>
+      <c r="G100" t="s">
         <v>313</v>
       </c>
-      <c r="G100" t="s">
+      <c r="H100" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>111</v>
       </c>
@@ -4313,19 +4626,22 @@
         <v>326</v>
       </c>
       <c r="D101" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E101" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F101" t="s">
+        <v>124</v>
+      </c>
+      <c r="G101" t="s">
         <v>314</v>
       </c>
-      <c r="G101" t="s">
+      <c r="H101" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>112</v>
       </c>
@@ -4336,15 +4652,18 @@
         <v>327</v>
       </c>
       <c r="D102" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E102" t="s">
-        <v>124</v>
+        <v>330</v>
       </c>
       <c r="F102" t="s">
+        <v>124</v>
+      </c>
+      <c r="G102" t="s">
         <v>315</v>
       </c>
-      <c r="G102" t="s">
+      <c r="H102" t="s">
         <v>93</v>
       </c>
     </row>

</xml_diff>